<commit_message>
adding more tests and more efficient code
</commit_message>
<xml_diff>
--- a/tests/files/experience/tables/graded_glm.xlsx
+++ b/tests/files/experience/tables/graded_glm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johnk\Desktop\github\morai\tests\files\experience\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22AAED3E-352B-48BD-863E-2ECC1C427D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF2CD67B-B7DB-4F46-9D19-787DD2242EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rate_table" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>constant</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>multiple * (1 - ['dummy'].clip(lower=0, upper=1))/(1-0) + 1 * (1-(1 -  ['dummy'].clip(lower=0, upper=1))/(1-0))</t>
+  </si>
+  <si>
+    <t>dummy</t>
   </si>
 </sst>
 </file>
@@ -444,10 +447,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -455,10 +458,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -466,10 +472,13 @@
         <v>3</v>
       </c>
       <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
         <v>7.1787645669163347E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -477,6 +486,9 @@
         <v>4</v>
       </c>
       <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>0.1082123543326768</v>
       </c>
     </row>

</xml_diff>